<commit_message>
feat: 增加读取部件参数蓝牙RSSI并优化CPU3菜单（CPU2 V1.15.0.0 / CPU3 V1.14.0.0）
版本：
- CPU2：V1.14.0.1 -> V1.15.0.0。
- CPU3：V1.13.0.0 -> V1.14.0.0。

协议版本/兼容性：
- 该历史提交未单列协议或兼容性说明；本次说明改写不改变该提交的文件树和程序行为。

本次修改：
- feat: 增加读取部件参数蓝牙RSSI并优化CPU3菜单

验证：
- py tools\check_wireless_rssi_contract.py
- py tools\check_si7000_protocol_contract.py
- py tools\check_density_level_control_contract.py
- py tools\check_read_part_params_refresh_contract.py
- py LTD_DISPLAY_CPU3\font_check.py
- py tools\update_flow_navigation.py
- cmake -S LTD_MAIN_CPU2 -B build\LTD_MAIN_CPU2 -G Ninja -DCMAKE_TOOLCHAIN_FILE=D:/CUBE/cmake/toolchain-arm-none-eabi.cmake
- cmake -S LTD_DISPLAY_CPU3 -B build\LTD_DISPLAY_CPU3 -G Ninja -DCMAKE_TOOLCHAIN_FILE=D:/CUBE/cmake/toolchain-arm-none-eabi.cmake
- cmake --build build\LTD_MAIN_CPU2
- cmake --build build\LTD_DISPLAY_CPU3
- git diff --cached --check
- py tools\check_version_bumped.py
</commit_message>
<xml_diff>
--- a/docs/04_界面与菜单/CPU3状态页显示参数矩阵.xlsx
+++ b/docs/04_界面与菜单/CPU3状态页显示参数矩阵.xlsx
@@ -687,7 +687,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -709,6 +709,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1122,12 +1128,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q74"/>
+  <dimension ref="A1:R74"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="16"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -1198,20 +1206,25 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>蓝牙RSSI</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>罐高</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>错误码</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>故障详情</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>MAC</t>
         </is>
@@ -1255,10 +1268,11 @@
       <c r="K2" s="6" t="inlineStr"/>
       <c r="L2" s="6" t="inlineStr"/>
       <c r="M2" s="6" t="inlineStr"/>
-      <c r="N2" s="6" t="inlineStr"/>
+      <c r="N2" s="8" t="n"/>
       <c r="O2" s="6" t="inlineStr"/>
       <c r="P2" s="6" t="inlineStr"/>
       <c r="Q2" s="6" t="inlineStr"/>
+      <c r="R2" s="6" t="inlineStr"/>
     </row>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -1298,10 +1312,11 @@
       <c r="K3" s="6" t="inlineStr"/>
       <c r="L3" s="6" t="inlineStr"/>
       <c r="M3" s="6" t="inlineStr"/>
-      <c r="N3" s="6" t="inlineStr"/>
+      <c r="N3" s="8" t="n"/>
       <c r="O3" s="6" t="inlineStr"/>
       <c r="P3" s="6" t="inlineStr"/>
       <c r="Q3" s="6" t="inlineStr"/>
+      <c r="R3" s="6" t="inlineStr"/>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -1345,10 +1360,11 @@
       <c r="K4" s="6" t="inlineStr"/>
       <c r="L4" s="6" t="inlineStr"/>
       <c r="M4" s="6" t="inlineStr"/>
-      <c r="N4" s="6" t="inlineStr"/>
+      <c r="N4" s="8" t="n"/>
       <c r="O4" s="6" t="inlineStr"/>
       <c r="P4" s="6" t="inlineStr"/>
       <c r="Q4" s="6" t="inlineStr"/>
+      <c r="R4" s="6" t="inlineStr"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -1388,10 +1404,11 @@
       <c r="K5" s="6" t="inlineStr"/>
       <c r="L5" s="6" t="inlineStr"/>
       <c r="M5" s="6" t="inlineStr"/>
-      <c r="N5" s="6" t="inlineStr"/>
+      <c r="N5" s="8" t="n"/>
       <c r="O5" s="6" t="inlineStr"/>
       <c r="P5" s="6" t="inlineStr"/>
       <c r="Q5" s="6" t="inlineStr"/>
+      <c r="R5" s="6" t="inlineStr"/>
     </row>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -1431,10 +1448,11 @@
       </c>
       <c r="L6" s="6" t="inlineStr"/>
       <c r="M6" s="6" t="inlineStr"/>
-      <c r="N6" s="6" t="inlineStr"/>
+      <c r="N6" s="8" t="n"/>
       <c r="O6" s="6" t="inlineStr"/>
       <c r="P6" s="6" t="inlineStr"/>
       <c r="Q6" s="6" t="inlineStr"/>
+      <c r="R6" s="6" t="inlineStr"/>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -1474,10 +1492,11 @@
       </c>
       <c r="L7" s="6" t="inlineStr"/>
       <c r="M7" s="6" t="inlineStr"/>
-      <c r="N7" s="6" t="inlineStr"/>
+      <c r="N7" s="8" t="n"/>
       <c r="O7" s="6" t="inlineStr"/>
       <c r="P7" s="6" t="inlineStr"/>
       <c r="Q7" s="6" t="inlineStr"/>
+      <c r="R7" s="6" t="inlineStr"/>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -1517,10 +1536,11 @@
       </c>
       <c r="L8" s="6" t="inlineStr"/>
       <c r="M8" s="6" t="inlineStr"/>
-      <c r="N8" s="6" t="inlineStr"/>
+      <c r="N8" s="8" t="n"/>
       <c r="O8" s="6" t="inlineStr"/>
       <c r="P8" s="6" t="inlineStr"/>
       <c r="Q8" s="6" t="inlineStr"/>
+      <c r="R8" s="6" t="inlineStr"/>
     </row>
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -1564,10 +1584,11 @@
       </c>
       <c r="L9" s="6" t="inlineStr"/>
       <c r="M9" s="6" t="inlineStr"/>
-      <c r="N9" s="6" t="inlineStr"/>
+      <c r="N9" s="8" t="n"/>
       <c r="O9" s="6" t="inlineStr"/>
       <c r="P9" s="6" t="inlineStr"/>
       <c r="Q9" s="6" t="inlineStr"/>
+      <c r="R9" s="6" t="inlineStr"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
@@ -1607,10 +1628,11 @@
       <c r="K10" s="6" t="inlineStr"/>
       <c r="L10" s="6" t="inlineStr"/>
       <c r="M10" s="6" t="inlineStr"/>
-      <c r="N10" s="6" t="inlineStr"/>
+      <c r="N10" s="8" t="n"/>
       <c r="O10" s="6" t="inlineStr"/>
       <c r="P10" s="6" t="inlineStr"/>
       <c r="Q10" s="6" t="inlineStr"/>
+      <c r="R10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
@@ -1650,10 +1672,11 @@
       <c r="K11" s="6" t="inlineStr"/>
       <c r="L11" s="6" t="inlineStr"/>
       <c r="M11" s="6" t="inlineStr"/>
-      <c r="N11" s="6" t="inlineStr"/>
+      <c r="N11" s="8" t="n"/>
       <c r="O11" s="6" t="inlineStr"/>
       <c r="P11" s="6" t="inlineStr"/>
       <c r="Q11" s="6" t="inlineStr"/>
+      <c r="R11" s="6" t="inlineStr"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
@@ -1697,10 +1720,11 @@
       <c r="K12" s="6" t="inlineStr"/>
       <c r="L12" s="6" t="inlineStr"/>
       <c r="M12" s="6" t="inlineStr"/>
-      <c r="N12" s="6" t="inlineStr"/>
+      <c r="N12" s="8" t="n"/>
       <c r="O12" s="6" t="inlineStr"/>
       <c r="P12" s="6" t="inlineStr"/>
       <c r="Q12" s="6" t="inlineStr"/>
+      <c r="R12" s="6" t="inlineStr"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -1744,10 +1768,11 @@
       <c r="K13" s="6" t="inlineStr"/>
       <c r="L13" s="6" t="inlineStr"/>
       <c r="M13" s="6" t="inlineStr"/>
-      <c r="N13" s="6" t="inlineStr"/>
+      <c r="N13" s="8" t="n"/>
       <c r="O13" s="6" t="inlineStr"/>
       <c r="P13" s="6" t="inlineStr"/>
       <c r="Q13" s="6" t="inlineStr"/>
+      <c r="R13" s="6" t="inlineStr"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -1791,10 +1816,11 @@
       <c r="K14" s="6" t="inlineStr"/>
       <c r="L14" s="6" t="inlineStr"/>
       <c r="M14" s="6" t="inlineStr"/>
-      <c r="N14" s="6" t="inlineStr"/>
+      <c r="N14" s="8" t="n"/>
       <c r="O14" s="6" t="inlineStr"/>
       <c r="P14" s="6" t="inlineStr"/>
       <c r="Q14" s="6" t="inlineStr"/>
+      <c r="R14" s="6" t="inlineStr"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -1838,10 +1864,11 @@
       <c r="K15" s="6" t="inlineStr"/>
       <c r="L15" s="6" t="inlineStr"/>
       <c r="M15" s="6" t="inlineStr"/>
-      <c r="N15" s="6" t="inlineStr"/>
+      <c r="N15" s="8" t="n"/>
       <c r="O15" s="6" t="inlineStr"/>
       <c r="P15" s="6" t="inlineStr"/>
       <c r="Q15" s="6" t="inlineStr"/>
+      <c r="R15" s="6" t="inlineStr"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -1877,10 +1904,11 @@
       <c r="K16" s="6" t="inlineStr"/>
       <c r="L16" s="6" t="inlineStr"/>
       <c r="M16" s="6" t="inlineStr"/>
-      <c r="N16" s="6" t="inlineStr"/>
+      <c r="N16" s="8" t="n"/>
       <c r="O16" s="6" t="inlineStr"/>
       <c r="P16" s="6" t="inlineStr"/>
       <c r="Q16" s="6" t="inlineStr"/>
+      <c r="R16" s="6" t="inlineStr"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -1916,10 +1944,11 @@
       <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr"/>
-      <c r="N17" s="6" t="inlineStr"/>
+      <c r="N17" s="8" t="n"/>
       <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="6" t="inlineStr"/>
       <c r="Q17" s="6" t="inlineStr"/>
+      <c r="R17" s="6" t="inlineStr"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
@@ -1955,10 +1984,11 @@
       <c r="K18" s="6" t="inlineStr"/>
       <c r="L18" s="6" t="inlineStr"/>
       <c r="M18" s="6" t="inlineStr"/>
-      <c r="N18" s="6" t="inlineStr"/>
+      <c r="N18" s="8" t="n"/>
       <c r="O18" s="6" t="inlineStr"/>
       <c r="P18" s="6" t="inlineStr"/>
       <c r="Q18" s="6" t="inlineStr"/>
+      <c r="R18" s="6" t="inlineStr"/>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
@@ -1994,10 +2024,11 @@
       <c r="K19" s="6" t="inlineStr"/>
       <c r="L19" s="6" t="inlineStr"/>
       <c r="M19" s="6" t="inlineStr"/>
-      <c r="N19" s="6" t="inlineStr"/>
+      <c r="N19" s="8" t="n"/>
       <c r="O19" s="6" t="inlineStr"/>
       <c r="P19" s="6" t="inlineStr"/>
       <c r="Q19" s="6" t="inlineStr"/>
+      <c r="R19" s="6" t="inlineStr"/>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
@@ -2033,10 +2064,11 @@
       <c r="K20" s="6" t="inlineStr"/>
       <c r="L20" s="6" t="inlineStr"/>
       <c r="M20" s="6" t="inlineStr"/>
-      <c r="N20" s="6" t="inlineStr"/>
+      <c r="N20" s="8" t="n"/>
       <c r="O20" s="6" t="inlineStr"/>
       <c r="P20" s="6" t="inlineStr"/>
       <c r="Q20" s="6" t="inlineStr"/>
+      <c r="R20" s="6" t="inlineStr"/>
     </row>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
@@ -2080,10 +2112,11 @@
       <c r="K21" s="6" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr"/>
       <c r="M21" s="6" t="inlineStr"/>
-      <c r="N21" s="6" t="inlineStr"/>
+      <c r="N21" s="8" t="n"/>
       <c r="O21" s="6" t="inlineStr"/>
       <c r="P21" s="6" t="inlineStr"/>
       <c r="Q21" s="6" t="inlineStr"/>
+      <c r="R21" s="6" t="inlineStr"/>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
@@ -2131,10 +2164,11 @@
       <c r="K22" s="6" t="inlineStr"/>
       <c r="L22" s="6" t="inlineStr"/>
       <c r="M22" s="6" t="inlineStr"/>
-      <c r="N22" s="6" t="inlineStr"/>
+      <c r="N22" s="8" t="n"/>
       <c r="O22" s="6" t="inlineStr"/>
       <c r="P22" s="6" t="inlineStr"/>
       <c r="Q22" s="6" t="inlineStr"/>
+      <c r="R22" s="6" t="inlineStr"/>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
@@ -2182,10 +2216,11 @@
       <c r="K23" s="6" t="inlineStr"/>
       <c r="L23" s="6" t="inlineStr"/>
       <c r="M23" s="6" t="inlineStr"/>
-      <c r="N23" s="6" t="inlineStr"/>
+      <c r="N23" s="8" t="n"/>
       <c r="O23" s="6" t="inlineStr"/>
       <c r="P23" s="6" t="inlineStr"/>
       <c r="Q23" s="6" t="inlineStr"/>
+      <c r="R23" s="6" t="inlineStr"/>
     </row>
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
@@ -2233,10 +2268,11 @@
       <c r="K24" s="6" t="inlineStr"/>
       <c r="L24" s="6" t="inlineStr"/>
       <c r="M24" s="6" t="inlineStr"/>
-      <c r="N24" s="6" t="inlineStr"/>
+      <c r="N24" s="8" t="n"/>
       <c r="O24" s="6" t="inlineStr"/>
       <c r="P24" s="6" t="inlineStr"/>
       <c r="Q24" s="6" t="inlineStr"/>
+      <c r="R24" s="6" t="inlineStr"/>
     </row>
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
@@ -2284,10 +2320,11 @@
       <c r="K25" s="6" t="inlineStr"/>
       <c r="L25" s="6" t="inlineStr"/>
       <c r="M25" s="6" t="inlineStr"/>
-      <c r="N25" s="6" t="inlineStr"/>
+      <c r="N25" s="8" t="n"/>
       <c r="O25" s="6" t="inlineStr"/>
       <c r="P25" s="6" t="inlineStr"/>
       <c r="Q25" s="6" t="inlineStr"/>
+      <c r="R25" s="6" t="inlineStr"/>
     </row>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
@@ -2335,10 +2372,11 @@
       <c r="K26" s="6" t="inlineStr"/>
       <c r="L26" s="6" t="inlineStr"/>
       <c r="M26" s="6" t="inlineStr"/>
-      <c r="N26" s="6" t="inlineStr"/>
+      <c r="N26" s="8" t="n"/>
       <c r="O26" s="6" t="inlineStr"/>
       <c r="P26" s="6" t="inlineStr"/>
       <c r="Q26" s="6" t="inlineStr"/>
+      <c r="R26" s="6" t="inlineStr"/>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
@@ -2374,10 +2412,11 @@
       <c r="K27" s="6" t="inlineStr"/>
       <c r="L27" s="6" t="inlineStr"/>
       <c r="M27" s="6" t="inlineStr"/>
-      <c r="N27" s="6" t="inlineStr"/>
+      <c r="N27" s="8" t="n"/>
       <c r="O27" s="6" t="inlineStr"/>
       <c r="P27" s="6" t="inlineStr"/>
       <c r="Q27" s="6" t="inlineStr"/>
+      <c r="R27" s="6" t="inlineStr"/>
     </row>
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
@@ -2429,10 +2468,11 @@
       <c r="K28" s="6" t="inlineStr"/>
       <c r="L28" s="6" t="inlineStr"/>
       <c r="M28" s="6" t="inlineStr"/>
-      <c r="N28" s="6" t="inlineStr"/>
+      <c r="N28" s="8" t="n"/>
       <c r="O28" s="6" t="inlineStr"/>
       <c r="P28" s="6" t="inlineStr"/>
       <c r="Q28" s="6" t="inlineStr"/>
+      <c r="R28" s="6" t="inlineStr"/>
     </row>
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
@@ -2476,10 +2516,11 @@
           <t>确认</t>
         </is>
       </c>
-      <c r="N29" s="6" t="inlineStr"/>
+      <c r="N29" s="9" t="n"/>
       <c r="O29" s="6" t="inlineStr"/>
       <c r="P29" s="6" t="inlineStr"/>
       <c r="Q29" s="6" t="inlineStr"/>
+      <c r="R29" s="6" t="inlineStr"/>
     </row>
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
@@ -2523,10 +2564,11 @@
           <t>确认</t>
         </is>
       </c>
-      <c r="N30" s="6" t="inlineStr"/>
+      <c r="N30" s="9" t="n"/>
       <c r="O30" s="6" t="inlineStr"/>
       <c r="P30" s="6" t="inlineStr"/>
       <c r="Q30" s="6" t="inlineStr"/>
+      <c r="R30" s="6" t="inlineStr"/>
     </row>
     <row r="31" ht="24" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
@@ -2570,14 +2612,15 @@
           <t>确认</t>
         </is>
       </c>
-      <c r="N31" s="5" t="inlineStr">
-        <is>
-          <t>确认</t>
-        </is>
-      </c>
-      <c r="O31" s="6" t="inlineStr"/>
+      <c r="N31" s="9" t="n"/>
+      <c r="O31" s="5" t="inlineStr">
+        <is>
+          <t>确认</t>
+        </is>
+      </c>
       <c r="P31" s="6" t="inlineStr"/>
       <c r="Q31" s="6" t="inlineStr"/>
+      <c r="R31" s="6" t="inlineStr"/>
     </row>
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="3" t="inlineStr">
@@ -2621,14 +2664,15 @@
           <t>确认</t>
         </is>
       </c>
-      <c r="N32" s="5" t="inlineStr">
-        <is>
-          <t>确认</t>
-        </is>
-      </c>
-      <c r="O32" s="6" t="inlineStr"/>
+      <c r="N32" s="9" t="n"/>
+      <c r="O32" s="5" t="inlineStr">
+        <is>
+          <t>确认</t>
+        </is>
+      </c>
       <c r="P32" s="6" t="inlineStr"/>
       <c r="Q32" s="6" t="inlineStr"/>
+      <c r="R32" s="6" t="inlineStr"/>
     </row>
     <row r="33" ht="24" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
@@ -2664,10 +2708,11 @@
       <c r="K33" s="6" t="inlineStr"/>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
-      <c r="N33" s="6" t="inlineStr"/>
+      <c r="N33" s="8" t="n"/>
       <c r="O33" s="6" t="inlineStr"/>
       <c r="P33" s="6" t="inlineStr"/>
       <c r="Q33" s="6" t="inlineStr"/>
+      <c r="R33" s="6" t="inlineStr"/>
     </row>
     <row r="34" ht="24" customHeight="1">
       <c r="A34" s="3" t="inlineStr">
@@ -2703,10 +2748,11 @@
       <c r="K34" s="6" t="inlineStr"/>
       <c r="L34" s="6" t="inlineStr"/>
       <c r="M34" s="6" t="inlineStr"/>
-      <c r="N34" s="6" t="inlineStr"/>
+      <c r="N34" s="8" t="n"/>
       <c r="O34" s="6" t="inlineStr"/>
       <c r="P34" s="6" t="inlineStr"/>
       <c r="Q34" s="6" t="inlineStr"/>
+      <c r="R34" s="6" t="inlineStr"/>
     </row>
     <row r="35" ht="24" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
@@ -2742,10 +2788,11 @@
       <c r="K35" s="6" t="inlineStr"/>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
-      <c r="N35" s="6" t="inlineStr"/>
+      <c r="N35" s="8" t="n"/>
       <c r="O35" s="6" t="inlineStr"/>
       <c r="P35" s="6" t="inlineStr"/>
       <c r="Q35" s="6" t="inlineStr"/>
+      <c r="R35" s="6" t="inlineStr"/>
     </row>
     <row r="36" ht="24" customHeight="1">
       <c r="A36" s="3" t="inlineStr">
@@ -2781,10 +2828,11 @@
       <c r="K36" s="6" t="inlineStr"/>
       <c r="L36" s="6" t="inlineStr"/>
       <c r="M36" s="6" t="inlineStr"/>
-      <c r="N36" s="6" t="inlineStr"/>
+      <c r="N36" s="8" t="n"/>
       <c r="O36" s="6" t="inlineStr"/>
       <c r="P36" s="6" t="inlineStr"/>
       <c r="Q36" s="6" t="inlineStr"/>
+      <c r="R36" s="6" t="inlineStr"/>
     </row>
     <row r="37" ht="24" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
@@ -2820,10 +2868,11 @@
       <c r="K37" s="6" t="inlineStr"/>
       <c r="L37" s="6" t="inlineStr"/>
       <c r="M37" s="6" t="inlineStr"/>
-      <c r="N37" s="6" t="inlineStr"/>
+      <c r="N37" s="8" t="n"/>
       <c r="O37" s="6" t="inlineStr"/>
       <c r="P37" s="6" t="inlineStr"/>
       <c r="Q37" s="6" t="inlineStr"/>
+      <c r="R37" s="6" t="inlineStr"/>
     </row>
     <row r="38" ht="24" customHeight="1">
       <c r="A38" s="3" t="inlineStr">
@@ -2859,10 +2908,11 @@
       <c r="K38" s="6" t="inlineStr"/>
       <c r="L38" s="6" t="inlineStr"/>
       <c r="M38" s="6" t="inlineStr"/>
-      <c r="N38" s="6" t="inlineStr"/>
+      <c r="N38" s="8" t="n"/>
       <c r="O38" s="6" t="inlineStr"/>
       <c r="P38" s="6" t="inlineStr"/>
       <c r="Q38" s="6" t="inlineStr"/>
+      <c r="R38" s="6" t="inlineStr"/>
     </row>
     <row r="39" ht="24" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
@@ -2898,10 +2948,11 @@
       <c r="K39" s="6" t="inlineStr"/>
       <c r="L39" s="6" t="inlineStr"/>
       <c r="M39" s="6" t="inlineStr"/>
-      <c r="N39" s="6" t="inlineStr"/>
+      <c r="N39" s="8" t="n"/>
       <c r="O39" s="6" t="inlineStr"/>
       <c r="P39" s="6" t="inlineStr"/>
       <c r="Q39" s="6" t="inlineStr"/>
+      <c r="R39" s="6" t="inlineStr"/>
     </row>
     <row r="40" ht="24" customHeight="1">
       <c r="A40" s="3" t="inlineStr">
@@ -2937,10 +2988,11 @@
       <c r="K40" s="6" t="inlineStr"/>
       <c r="L40" s="6" t="inlineStr"/>
       <c r="M40" s="6" t="inlineStr"/>
-      <c r="N40" s="6" t="inlineStr"/>
+      <c r="N40" s="8" t="n"/>
       <c r="O40" s="6" t="inlineStr"/>
       <c r="P40" s="6" t="inlineStr"/>
       <c r="Q40" s="6" t="inlineStr"/>
+      <c r="R40" s="6" t="inlineStr"/>
     </row>
     <row r="41" ht="24" customHeight="1">
       <c r="A41" s="3" t="inlineStr">
@@ -2976,10 +3028,11 @@
       <c r="K41" s="6" t="inlineStr"/>
       <c r="L41" s="6" t="inlineStr"/>
       <c r="M41" s="6" t="inlineStr"/>
-      <c r="N41" s="6" t="inlineStr"/>
+      <c r="N41" s="8" t="n"/>
       <c r="O41" s="6" t="inlineStr"/>
       <c r="P41" s="6" t="inlineStr"/>
       <c r="Q41" s="6" t="inlineStr"/>
+      <c r="R41" s="6" t="inlineStr"/>
     </row>
     <row r="42" ht="24" customHeight="1">
       <c r="A42" s="3" t="inlineStr">
@@ -3015,10 +3068,11 @@
       <c r="K42" s="6" t="inlineStr"/>
       <c r="L42" s="6" t="inlineStr"/>
       <c r="M42" s="6" t="inlineStr"/>
-      <c r="N42" s="6" t="inlineStr"/>
+      <c r="N42" s="8" t="n"/>
       <c r="O42" s="6" t="inlineStr"/>
       <c r="P42" s="6" t="inlineStr"/>
       <c r="Q42" s="6" t="inlineStr"/>
+      <c r="R42" s="6" t="inlineStr"/>
     </row>
     <row r="43" ht="24" customHeight="1">
       <c r="A43" s="3" t="inlineStr">
@@ -3054,10 +3108,11 @@
       <c r="K43" s="6" t="inlineStr"/>
       <c r="L43" s="6" t="inlineStr"/>
       <c r="M43" s="6" t="inlineStr"/>
-      <c r="N43" s="6" t="inlineStr"/>
+      <c r="N43" s="8" t="n"/>
       <c r="O43" s="6" t="inlineStr"/>
       <c r="P43" s="6" t="inlineStr"/>
       <c r="Q43" s="6" t="inlineStr"/>
+      <c r="R43" s="6" t="inlineStr"/>
     </row>
     <row r="44" ht="24" customHeight="1">
       <c r="A44" s="3" t="inlineStr">
@@ -3093,10 +3148,11 @@
       <c r="K44" s="6" t="inlineStr"/>
       <c r="L44" s="6" t="inlineStr"/>
       <c r="M44" s="6" t="inlineStr"/>
-      <c r="N44" s="6" t="inlineStr"/>
+      <c r="N44" s="8" t="n"/>
       <c r="O44" s="6" t="inlineStr"/>
       <c r="P44" s="6" t="inlineStr"/>
       <c r="Q44" s="6" t="inlineStr"/>
+      <c r="R44" s="6" t="inlineStr"/>
     </row>
     <row r="45" ht="24" customHeight="1">
       <c r="A45" s="3" t="inlineStr">
@@ -3132,10 +3188,11 @@
       <c r="K45" s="6" t="inlineStr"/>
       <c r="L45" s="6" t="inlineStr"/>
       <c r="M45" s="6" t="inlineStr"/>
-      <c r="N45" s="6" t="inlineStr"/>
+      <c r="N45" s="8" t="n"/>
       <c r="O45" s="6" t="inlineStr"/>
       <c r="P45" s="6" t="inlineStr"/>
       <c r="Q45" s="6" t="inlineStr"/>
+      <c r="R45" s="6" t="inlineStr"/>
     </row>
     <row r="46" ht="24" customHeight="1">
       <c r="A46" s="3" t="inlineStr">
@@ -3171,10 +3228,11 @@
       <c r="K46" s="6" t="inlineStr"/>
       <c r="L46" s="6" t="inlineStr"/>
       <c r="M46" s="6" t="inlineStr"/>
-      <c r="N46" s="6" t="inlineStr"/>
+      <c r="N46" s="8" t="n"/>
       <c r="O46" s="6" t="inlineStr"/>
       <c r="P46" s="6" t="inlineStr"/>
       <c r="Q46" s="6" t="inlineStr"/>
+      <c r="R46" s="6" t="inlineStr"/>
     </row>
     <row r="47" ht="24" customHeight="1">
       <c r="A47" s="3" t="inlineStr">
@@ -3210,10 +3268,11 @@
       <c r="K47" s="6" t="inlineStr"/>
       <c r="L47" s="6" t="inlineStr"/>
       <c r="M47" s="6" t="inlineStr"/>
-      <c r="N47" s="6" t="inlineStr"/>
+      <c r="N47" s="8" t="n"/>
       <c r="O47" s="6" t="inlineStr"/>
       <c r="P47" s="6" t="inlineStr"/>
       <c r="Q47" s="6" t="inlineStr"/>
+      <c r="R47" s="6" t="inlineStr"/>
     </row>
     <row r="48" ht="24" customHeight="1">
       <c r="A48" s="3" t="inlineStr">
@@ -3249,10 +3308,11 @@
       <c r="K48" s="6" t="inlineStr"/>
       <c r="L48" s="6" t="inlineStr"/>
       <c r="M48" s="6" t="inlineStr"/>
-      <c r="N48" s="6" t="inlineStr"/>
+      <c r="N48" s="8" t="n"/>
       <c r="O48" s="6" t="inlineStr"/>
       <c r="P48" s="6" t="inlineStr"/>
       <c r="Q48" s="6" t="inlineStr"/>
+      <c r="R48" s="6" t="inlineStr"/>
     </row>
     <row r="49" ht="24" customHeight="1">
       <c r="A49" s="3" t="inlineStr">
@@ -3288,10 +3348,11 @@
       <c r="K49" s="6" t="inlineStr"/>
       <c r="L49" s="6" t="inlineStr"/>
       <c r="M49" s="6" t="inlineStr"/>
-      <c r="N49" s="6" t="inlineStr"/>
+      <c r="N49" s="8" t="n"/>
       <c r="O49" s="6" t="inlineStr"/>
       <c r="P49" s="6" t="inlineStr"/>
       <c r="Q49" s="6" t="inlineStr"/>
+      <c r="R49" s="6" t="inlineStr"/>
     </row>
     <row r="50" ht="24" customHeight="1">
       <c r="A50" s="3" t="inlineStr">
@@ -3327,10 +3388,11 @@
       <c r="K50" s="6" t="inlineStr"/>
       <c r="L50" s="6" t="inlineStr"/>
       <c r="M50" s="6" t="inlineStr"/>
-      <c r="N50" s="6" t="inlineStr"/>
+      <c r="N50" s="8" t="n"/>
       <c r="O50" s="6" t="inlineStr"/>
       <c r="P50" s="6" t="inlineStr"/>
       <c r="Q50" s="6" t="inlineStr"/>
+      <c r="R50" s="6" t="inlineStr"/>
     </row>
     <row r="51" ht="24" customHeight="1">
       <c r="A51" s="3" t="inlineStr">
@@ -3366,10 +3428,11 @@
       <c r="K51" s="6" t="inlineStr"/>
       <c r="L51" s="6" t="inlineStr"/>
       <c r="M51" s="6" t="inlineStr"/>
-      <c r="N51" s="6" t="inlineStr"/>
+      <c r="N51" s="8" t="n"/>
       <c r="O51" s="6" t="inlineStr"/>
       <c r="P51" s="6" t="inlineStr"/>
       <c r="Q51" s="6" t="inlineStr"/>
+      <c r="R51" s="6" t="inlineStr"/>
     </row>
     <row r="52" ht="24" customHeight="1">
       <c r="A52" s="3" t="inlineStr">
@@ -3405,10 +3468,11 @@
       <c r="K52" s="6" t="inlineStr"/>
       <c r="L52" s="6" t="inlineStr"/>
       <c r="M52" s="6" t="inlineStr"/>
-      <c r="N52" s="6" t="inlineStr"/>
+      <c r="N52" s="8" t="n"/>
       <c r="O52" s="6" t="inlineStr"/>
       <c r="P52" s="6" t="inlineStr"/>
       <c r="Q52" s="6" t="inlineStr"/>
+      <c r="R52" s="6" t="inlineStr"/>
     </row>
     <row r="53" ht="24" customHeight="1">
       <c r="A53" s="3" t="inlineStr">
@@ -3444,18 +3508,19 @@
       <c r="K53" s="6" t="inlineStr"/>
       <c r="L53" s="6" t="inlineStr"/>
       <c r="M53" s="6" t="inlineStr"/>
-      <c r="N53" s="6" t="inlineStr"/>
-      <c r="O53" s="5" t="inlineStr">
-        <is>
-          <t>确认</t>
-        </is>
-      </c>
+      <c r="N53" s="8" t="n"/>
+      <c r="O53" s="6" t="inlineStr"/>
       <c r="P53" s="5" t="inlineStr">
         <is>
           <t>确认</t>
         </is>
       </c>
-      <c r="Q53" s="6" t="inlineStr"/>
+      <c r="Q53" s="5" t="inlineStr">
+        <is>
+          <t>确认</t>
+        </is>
+      </c>
+      <c r="R53" s="6" t="inlineStr"/>
     </row>
     <row r="54" ht="24" customHeight="1">
       <c r="A54" s="3" t="inlineStr">
@@ -3483,10 +3548,11 @@
       <c r="K54" s="6" t="inlineStr"/>
       <c r="L54" s="6" t="inlineStr"/>
       <c r="M54" s="6" t="inlineStr"/>
-      <c r="N54" s="6" t="inlineStr"/>
+      <c r="N54" s="8" t="n"/>
       <c r="O54" s="6" t="inlineStr"/>
       <c r="P54" s="6" t="inlineStr"/>
       <c r="Q54" s="6" t="inlineStr"/>
+      <c r="R54" s="6" t="inlineStr"/>
     </row>
     <row r="55" ht="24" customHeight="1">
       <c r="A55" s="3" t="inlineStr">
@@ -3514,10 +3580,11 @@
       <c r="K55" s="6" t="inlineStr"/>
       <c r="L55" s="6" t="inlineStr"/>
       <c r="M55" s="6" t="inlineStr"/>
-      <c r="N55" s="6" t="inlineStr"/>
+      <c r="N55" s="8" t="n"/>
       <c r="O55" s="6" t="inlineStr"/>
       <c r="P55" s="6" t="inlineStr"/>
-      <c r="Q55" s="5" t="inlineStr">
+      <c r="Q55" s="6" t="inlineStr"/>
+      <c r="R55" s="5" t="inlineStr">
         <is>
           <t>确认</t>
         </is>
@@ -3557,10 +3624,11 @@
       <c r="K56" s="6" t="inlineStr"/>
       <c r="L56" s="6" t="inlineStr"/>
       <c r="M56" s="6" t="inlineStr"/>
-      <c r="N56" s="6" t="inlineStr"/>
+      <c r="N56" s="8" t="n"/>
       <c r="O56" s="6" t="inlineStr"/>
       <c r="P56" s="6" t="inlineStr"/>
       <c r="Q56" s="6" t="inlineStr"/>
+      <c r="R56" s="6" t="inlineStr"/>
     </row>
     <row r="57" ht="24" customHeight="1">
       <c r="A57" s="3" t="inlineStr">
@@ -3596,10 +3664,11 @@
       <c r="K57" s="6" t="inlineStr"/>
       <c r="L57" s="6" t="inlineStr"/>
       <c r="M57" s="6" t="inlineStr"/>
-      <c r="N57" s="6" t="inlineStr"/>
+      <c r="N57" s="8" t="n"/>
       <c r="O57" s="6" t="inlineStr"/>
       <c r="P57" s="6" t="inlineStr"/>
       <c r="Q57" s="6" t="inlineStr"/>
+      <c r="R57" s="6" t="inlineStr"/>
     </row>
     <row r="58" ht="24" customHeight="1">
       <c r="A58" s="3" t="inlineStr">
@@ -3635,10 +3704,11 @@
       <c r="K58" s="6" t="inlineStr"/>
       <c r="L58" s="6" t="inlineStr"/>
       <c r="M58" s="6" t="inlineStr"/>
-      <c r="N58" s="6" t="inlineStr"/>
+      <c r="N58" s="8" t="n"/>
       <c r="O58" s="6" t="inlineStr"/>
       <c r="P58" s="6" t="inlineStr"/>
       <c r="Q58" s="6" t="inlineStr"/>
+      <c r="R58" s="6" t="inlineStr"/>
     </row>
     <row r="59" ht="24" customHeight="1">
       <c r="A59" s="3" t="inlineStr">
@@ -3674,10 +3744,11 @@
       <c r="K59" s="6" t="inlineStr"/>
       <c r="L59" s="6" t="inlineStr"/>
       <c r="M59" s="6" t="inlineStr"/>
-      <c r="N59" s="6" t="inlineStr"/>
+      <c r="N59" s="8" t="n"/>
       <c r="O59" s="6" t="inlineStr"/>
       <c r="P59" s="6" t="inlineStr"/>
       <c r="Q59" s="6" t="inlineStr"/>
+      <c r="R59" s="6" t="inlineStr"/>
     </row>
     <row r="60" ht="24" customHeight="1">
       <c r="A60" s="3" t="inlineStr">
@@ -3713,10 +3784,11 @@
       <c r="K60" s="6" t="inlineStr"/>
       <c r="L60" s="6" t="inlineStr"/>
       <c r="M60" s="6" t="inlineStr"/>
-      <c r="N60" s="6" t="inlineStr"/>
+      <c r="N60" s="8" t="n"/>
       <c r="O60" s="6" t="inlineStr"/>
       <c r="P60" s="6" t="inlineStr"/>
       <c r="Q60" s="6" t="inlineStr"/>
+      <c r="R60" s="6" t="inlineStr"/>
     </row>
     <row r="61" ht="24" customHeight="1">
       <c r="A61" s="3" t="inlineStr">
@@ -3752,10 +3824,11 @@
       <c r="K61" s="6" t="inlineStr"/>
       <c r="L61" s="6" t="inlineStr"/>
       <c r="M61" s="6" t="inlineStr"/>
-      <c r="N61" s="6" t="inlineStr"/>
+      <c r="N61" s="8" t="n"/>
       <c r="O61" s="6" t="inlineStr"/>
       <c r="P61" s="6" t="inlineStr"/>
       <c r="Q61" s="6" t="inlineStr"/>
+      <c r="R61" s="6" t="inlineStr"/>
     </row>
     <row r="62" ht="24" customHeight="1">
       <c r="A62" s="3" t="inlineStr">
@@ -3791,10 +3864,11 @@
       <c r="K62" s="6" t="inlineStr"/>
       <c r="L62" s="6" t="inlineStr"/>
       <c r="M62" s="6" t="inlineStr"/>
-      <c r="N62" s="6" t="inlineStr"/>
+      <c r="N62" s="8" t="n"/>
       <c r="O62" s="6" t="inlineStr"/>
       <c r="P62" s="6" t="inlineStr"/>
       <c r="Q62" s="6" t="inlineStr"/>
+      <c r="R62" s="6" t="inlineStr"/>
     </row>
     <row r="63" ht="24" customHeight="1">
       <c r="A63" s="3" t="inlineStr">
@@ -3830,10 +3904,11 @@
       <c r="K63" s="6" t="inlineStr"/>
       <c r="L63" s="6" t="inlineStr"/>
       <c r="M63" s="6" t="inlineStr"/>
-      <c r="N63" s="6" t="inlineStr"/>
+      <c r="N63" s="8" t="n"/>
       <c r="O63" s="6" t="inlineStr"/>
       <c r="P63" s="6" t="inlineStr"/>
       <c r="Q63" s="6" t="inlineStr"/>
+      <c r="R63" s="6" t="inlineStr"/>
     </row>
     <row r="64" ht="24" customHeight="1">
       <c r="A64" s="3" t="inlineStr">
@@ -3869,10 +3944,11 @@
       <c r="K64" s="6" t="inlineStr"/>
       <c r="L64" s="6" t="inlineStr"/>
       <c r="M64" s="6" t="inlineStr"/>
-      <c r="N64" s="6" t="inlineStr"/>
+      <c r="N64" s="8" t="n"/>
       <c r="O64" s="6" t="inlineStr"/>
       <c r="P64" s="6" t="inlineStr"/>
       <c r="Q64" s="6" t="inlineStr"/>
+      <c r="R64" s="6" t="inlineStr"/>
     </row>
     <row r="65" ht="24" customHeight="1">
       <c r="A65" s="3" t="inlineStr">
@@ -3908,10 +3984,11 @@
       <c r="K65" s="6" t="inlineStr"/>
       <c r="L65" s="6" t="inlineStr"/>
       <c r="M65" s="6" t="inlineStr"/>
-      <c r="N65" s="6" t="inlineStr"/>
+      <c r="N65" s="8" t="n"/>
       <c r="O65" s="6" t="inlineStr"/>
       <c r="P65" s="6" t="inlineStr"/>
       <c r="Q65" s="6" t="inlineStr"/>
+      <c r="R65" s="6" t="inlineStr"/>
     </row>
     <row r="66" ht="24" customHeight="1">
       <c r="A66" s="3" t="inlineStr">
@@ -3947,10 +4024,11 @@
       <c r="K66" s="6" t="inlineStr"/>
       <c r="L66" s="6" t="inlineStr"/>
       <c r="M66" s="6" t="inlineStr"/>
-      <c r="N66" s="6" t="inlineStr"/>
+      <c r="N66" s="8" t="n"/>
       <c r="O66" s="6" t="inlineStr"/>
       <c r="P66" s="6" t="inlineStr"/>
       <c r="Q66" s="6" t="inlineStr"/>
+      <c r="R66" s="6" t="inlineStr"/>
     </row>
     <row r="67" ht="24" customHeight="1">
       <c r="A67" s="3" t="inlineStr">
@@ -3986,10 +4064,11 @@
       <c r="K67" s="6" t="inlineStr"/>
       <c r="L67" s="6" t="inlineStr"/>
       <c r="M67" s="6" t="inlineStr"/>
-      <c r="N67" s="6" t="inlineStr"/>
+      <c r="N67" s="8" t="n"/>
       <c r="O67" s="6" t="inlineStr"/>
       <c r="P67" s="6" t="inlineStr"/>
       <c r="Q67" s="6" t="inlineStr"/>
+      <c r="R67" s="6" t="inlineStr"/>
     </row>
     <row r="68" ht="24" customHeight="1">
       <c r="A68" s="3" t="inlineStr">
@@ -4017,21 +4096,9 @@
           <t>确认</t>
         </is>
       </c>
-      <c r="F68" s="5" t="inlineStr">
-        <is>
-          <t>确认</t>
-        </is>
-      </c>
-      <c r="G68" s="5" t="inlineStr">
-        <is>
-          <t>确认</t>
-        </is>
-      </c>
-      <c r="H68" s="5" t="inlineStr">
-        <is>
-          <t>确认</t>
-        </is>
-      </c>
+      <c r="F68" s="5" t="n"/>
+      <c r="G68" s="5" t="n"/>
+      <c r="H68" s="5" t="n"/>
       <c r="I68" s="5" t="inlineStr">
         <is>
           <t>确认</t>
@@ -4057,14 +4124,15 @@
           <t>确认</t>
         </is>
       </c>
-      <c r="N68" s="5" t="inlineStr">
-        <is>
-          <t>确认</t>
-        </is>
-      </c>
-      <c r="O68" s="6" t="inlineStr"/>
-      <c r="P68" s="6" t="inlineStr"/>
-      <c r="Q68" s="6" t="inlineStr"/>
+      <c r="N68" s="9" t="inlineStr">
+        <is>
+          <t>确认</t>
+        </is>
+      </c>
+      <c r="O68" s="5" t="n"/>
+      <c r="P68" s="6" t="n"/>
+      <c r="Q68" s="6" t="n"/>
+      <c r="R68" s="6" t="n"/>
     </row>
     <row r="69" ht="24" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
@@ -4100,10 +4168,11 @@
       <c r="K69" s="6" t="inlineStr"/>
       <c r="L69" s="6" t="inlineStr"/>
       <c r="M69" s="6" t="inlineStr"/>
-      <c r="N69" s="6" t="inlineStr"/>
+      <c r="N69" s="8" t="n"/>
       <c r="O69" s="6" t="inlineStr"/>
       <c r="P69" s="6" t="inlineStr"/>
       <c r="Q69" s="6" t="inlineStr"/>
+      <c r="R69" s="6" t="inlineStr"/>
     </row>
     <row r="70" ht="24" customHeight="1">
       <c r="A70" s="3" t="inlineStr">
@@ -4139,10 +4208,11 @@
       <c r="K70" s="6" t="inlineStr"/>
       <c r="L70" s="6" t="inlineStr"/>
       <c r="M70" s="6" t="inlineStr"/>
-      <c r="N70" s="6" t="inlineStr"/>
+      <c r="N70" s="8" t="n"/>
       <c r="O70" s="6" t="inlineStr"/>
       <c r="P70" s="6" t="inlineStr"/>
       <c r="Q70" s="6" t="inlineStr"/>
+      <c r="R70" s="6" t="inlineStr"/>
     </row>
     <row r="71" ht="24" customHeight="1">
       <c r="A71" s="3" t="inlineStr">
@@ -4178,10 +4248,11 @@
       <c r="K71" s="6" t="inlineStr"/>
       <c r="L71" s="6" t="inlineStr"/>
       <c r="M71" s="6" t="inlineStr"/>
-      <c r="N71" s="6" t="inlineStr"/>
+      <c r="N71" s="8" t="n"/>
       <c r="O71" s="6" t="inlineStr"/>
       <c r="P71" s="6" t="inlineStr"/>
       <c r="Q71" s="6" t="inlineStr"/>
+      <c r="R71" s="6" t="inlineStr"/>
     </row>
     <row r="72" ht="24" customHeight="1">
       <c r="A72" s="3" t="inlineStr">
@@ -4217,10 +4288,11 @@
       <c r="K72" s="6" t="inlineStr"/>
       <c r="L72" s="6" t="inlineStr"/>
       <c r="M72" s="6" t="inlineStr"/>
-      <c r="N72" s="6" t="inlineStr"/>
+      <c r="N72" s="8" t="n"/>
       <c r="O72" s="6" t="inlineStr"/>
       <c r="P72" s="6" t="inlineStr"/>
       <c r="Q72" s="6" t="inlineStr"/>
+      <c r="R72" s="6" t="inlineStr"/>
     </row>
     <row r="73" ht="24" customHeight="1">
       <c r="A73" s="3" t="inlineStr">
@@ -4256,10 +4328,11 @@
       <c r="K73" s="6" t="inlineStr"/>
       <c r="L73" s="6" t="inlineStr"/>
       <c r="M73" s="6" t="inlineStr"/>
-      <c r="N73" s="6" t="inlineStr"/>
+      <c r="N73" s="8" t="n"/>
       <c r="O73" s="6" t="inlineStr"/>
       <c r="P73" s="6" t="inlineStr"/>
       <c r="Q73" s="6" t="inlineStr"/>
+      <c r="R73" s="6" t="inlineStr"/>
     </row>
     <row r="74" ht="24" customHeight="1">
       <c r="A74" s="3" t="inlineStr">
@@ -4295,10 +4368,11 @@
       <c r="K74" s="6" t="inlineStr"/>
       <c r="L74" s="6" t="inlineStr"/>
       <c r="M74" s="6" t="inlineStr"/>
-      <c r="N74" s="6" t="inlineStr"/>
+      <c r="N74" s="8" t="n"/>
       <c r="O74" s="6" t="inlineStr"/>
       <c r="P74" s="6" t="inlineStr"/>
       <c r="Q74" s="6" t="inlineStr"/>
+      <c r="R74" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Q74"/>
@@ -4312,7 +4386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V74"/>
+  <dimension ref="A1:W74"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4322,6 +4396,8 @@
     <col width="44" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="21"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4417,20 +4493,25 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
+          <t>蓝牙RSSI</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>罐高</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>错误码</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>故障详情</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>MAC</t>
         </is>
@@ -4499,10 +4580,11 @@
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
       <c r="R2" s="2" t="inlineStr"/>
-      <c r="S2" s="2" t="inlineStr"/>
+      <c r="S2" s="7" t="n"/>
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="inlineStr"/>
+      <c r="W2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="54" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -4567,10 +4649,11 @@
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
       <c r="R3" s="2" t="inlineStr"/>
-      <c r="S3" s="2" t="inlineStr"/>
+      <c r="S3" s="7" t="n"/>
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="inlineStr"/>
+      <c r="W3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="40.5" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -4639,10 +4722,11 @@
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="inlineStr"/>
-      <c r="S4" s="2" t="inlineStr"/>
+      <c r="S4" s="7" t="n"/>
       <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="inlineStr"/>
+      <c r="W4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="27" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -4707,10 +4791,11 @@
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="inlineStr"/>
-      <c r="S5" s="2" t="inlineStr"/>
+      <c r="S5" s="7" t="n"/>
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="inlineStr"/>
+      <c r="W5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="27" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -4775,10 +4860,11 @@
       </c>
       <c r="Q6" s="2" t="inlineStr"/>
       <c r="R6" s="2" t="inlineStr"/>
-      <c r="S6" s="2" t="inlineStr"/>
+      <c r="S6" s="7" t="n"/>
       <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="inlineStr"/>
+      <c r="W6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="27" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -4843,10 +4929,11 @@
       </c>
       <c r="Q7" s="2" t="inlineStr"/>
       <c r="R7" s="2" t="inlineStr"/>
-      <c r="S7" s="2" t="inlineStr"/>
+      <c r="S7" s="7" t="n"/>
       <c r="T7" s="2" t="inlineStr"/>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="inlineStr"/>
+      <c r="W7" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="27" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -4911,10 +4998,11 @@
       </c>
       <c r="Q8" s="2" t="inlineStr"/>
       <c r="R8" s="2" t="inlineStr"/>
-      <c r="S8" s="2" t="inlineStr"/>
+      <c r="S8" s="7" t="n"/>
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="inlineStr"/>
+      <c r="W8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="40.5" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -4983,10 +5071,11 @@
       </c>
       <c r="Q9" s="2" t="inlineStr"/>
       <c r="R9" s="2" t="inlineStr"/>
-      <c r="S9" s="2" t="inlineStr"/>
+      <c r="S9" s="7" t="n"/>
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="inlineStr"/>
+      <c r="W9" s="2" t="inlineStr"/>
     </row>
     <row r="10" ht="27" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
@@ -5051,10 +5140,11 @@
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
       <c r="R10" s="2" t="inlineStr"/>
-      <c r="S10" s="2" t="inlineStr"/>
+      <c r="S10" s="7" t="n"/>
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="inlineStr"/>
+      <c r="W10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="27" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
@@ -5119,10 +5209,11 @@
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
       <c r="R11" s="2" t="inlineStr"/>
-      <c r="S11" s="2" t="inlineStr"/>
+      <c r="S11" s="7" t="n"/>
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="inlineStr"/>
+      <c r="W11" s="2" t="inlineStr"/>
     </row>
     <row r="12" ht="40.5" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
@@ -5191,10 +5282,11 @@
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="inlineStr"/>
-      <c r="S12" s="2" t="inlineStr"/>
+      <c r="S12" s="7" t="n"/>
       <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="inlineStr"/>
+      <c r="W12" s="2" t="inlineStr"/>
     </row>
     <row r="13" ht="40.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -5263,10 +5355,11 @@
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
       <c r="R13" s="2" t="inlineStr"/>
-      <c r="S13" s="2" t="inlineStr"/>
+      <c r="S13" s="7" t="n"/>
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="inlineStr"/>
+      <c r="W13" s="2" t="inlineStr"/>
     </row>
     <row r="14" ht="54" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -5335,10 +5428,11 @@
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
       <c r="R14" s="2" t="inlineStr"/>
-      <c r="S14" s="2" t="inlineStr"/>
+      <c r="S14" s="7" t="n"/>
       <c r="T14" s="2" t="inlineStr"/>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="inlineStr"/>
+      <c r="W14" s="2" t="inlineStr"/>
     </row>
     <row r="15" ht="54" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -5407,10 +5501,11 @@
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
       <c r="R15" s="2" t="inlineStr"/>
-      <c r="S15" s="2" t="inlineStr"/>
+      <c r="S15" s="7" t="n"/>
       <c r="T15" s="2" t="inlineStr"/>
       <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="inlineStr"/>
+      <c r="W15" s="2" t="inlineStr"/>
     </row>
     <row r="16" ht="27" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -5471,10 +5566,11 @@
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
       <c r="R16" s="2" t="inlineStr"/>
-      <c r="S16" s="2" t="inlineStr"/>
+      <c r="S16" s="7" t="n"/>
       <c r="T16" s="2" t="inlineStr"/>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="inlineStr"/>
+      <c r="W16" s="2" t="inlineStr"/>
     </row>
     <row r="17" ht="27" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -5535,10 +5631,11 @@
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
       <c r="R17" s="2" t="inlineStr"/>
-      <c r="S17" s="2" t="inlineStr"/>
+      <c r="S17" s="7" t="n"/>
       <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="inlineStr"/>
+      <c r="W17" s="2" t="inlineStr"/>
     </row>
     <row r="18" ht="27" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
@@ -5599,10 +5696,11 @@
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
       <c r="R18" s="2" t="inlineStr"/>
-      <c r="S18" s="2" t="inlineStr"/>
+      <c r="S18" s="7" t="n"/>
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="inlineStr"/>
+      <c r="W18" s="2" t="inlineStr"/>
     </row>
     <row r="19" ht="27" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
@@ -5663,10 +5761,11 @@
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
       <c r="R19" s="2" t="inlineStr"/>
-      <c r="S19" s="2" t="inlineStr"/>
+      <c r="S19" s="7" t="n"/>
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="inlineStr"/>
+      <c r="W19" s="2" t="inlineStr"/>
     </row>
     <row r="20" ht="27" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
@@ -5727,10 +5826,11 @@
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="inlineStr"/>
-      <c r="S20" s="2" t="inlineStr"/>
+      <c r="S20" s="7" t="n"/>
       <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="inlineStr"/>
+      <c r="W20" s="2" t="inlineStr"/>
     </row>
     <row r="21" ht="27" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
@@ -5799,10 +5899,11 @@
       <c r="P21" s="2" t="n"/>
       <c r="Q21" s="2" t="n"/>
       <c r="R21" s="2" t="n"/>
-      <c r="S21" s="2" t="n"/>
+      <c r="S21" s="7" t="n"/>
       <c r="T21" s="2" t="n"/>
       <c r="U21" s="2" t="n"/>
       <c r="V21" s="2" t="n"/>
+      <c r="W21" s="2" t="n"/>
     </row>
     <row r="22" ht="27" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
@@ -5875,10 +5976,11 @@
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="inlineStr"/>
-      <c r="S22" s="2" t="inlineStr"/>
+      <c r="S22" s="7" t="n"/>
       <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="inlineStr"/>
+      <c r="W22" s="2" t="inlineStr"/>
     </row>
     <row r="23" ht="27" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
@@ -5951,10 +6053,11 @@
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
       <c r="R23" s="2" t="inlineStr"/>
-      <c r="S23" s="2" t="inlineStr"/>
+      <c r="S23" s="7" t="n"/>
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="inlineStr"/>
+      <c r="W23" s="2" t="inlineStr"/>
     </row>
     <row r="24" ht="27" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
@@ -6027,10 +6130,11 @@
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
       <c r="R24" s="2" t="inlineStr"/>
-      <c r="S24" s="2" t="inlineStr"/>
+      <c r="S24" s="7" t="n"/>
       <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="inlineStr"/>
+      <c r="W24" s="2" t="inlineStr"/>
     </row>
     <row r="25" ht="27" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
@@ -6103,10 +6207,11 @@
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
       <c r="R25" s="2" t="inlineStr"/>
-      <c r="S25" s="2" t="inlineStr"/>
+      <c r="S25" s="7" t="n"/>
       <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="inlineStr"/>
+      <c r="W25" s="2" t="inlineStr"/>
     </row>
     <row r="26" ht="27" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
@@ -6179,10 +6284,11 @@
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
       <c r="R26" s="2" t="inlineStr"/>
-      <c r="S26" s="2" t="inlineStr"/>
+      <c r="S26" s="7" t="n"/>
       <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="inlineStr"/>
+      <c r="W26" s="2" t="inlineStr"/>
     </row>
     <row r="27" ht="27" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
@@ -6243,10 +6349,11 @@
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
       <c r="R27" s="2" t="inlineStr"/>
-      <c r="S27" s="2" t="inlineStr"/>
+      <c r="S27" s="7" t="n"/>
       <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="inlineStr"/>
+      <c r="W27" s="2" t="inlineStr"/>
     </row>
     <row r="28" ht="54" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
@@ -6323,10 +6430,11 @@
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
       <c r="R28" s="2" t="inlineStr"/>
-      <c r="S28" s="2" t="inlineStr"/>
+      <c r="S28" s="7" t="n"/>
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="inlineStr"/>
+      <c r="W28" s="2" t="inlineStr"/>
     </row>
     <row r="29" ht="40.5" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
@@ -6395,10 +6503,11 @@
           <t>确认</t>
         </is>
       </c>
-      <c r="S29" s="2" t="inlineStr"/>
+      <c r="S29" s="9" t="n"/>
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="inlineStr"/>
+      <c r="W29" s="2" t="inlineStr"/>
     </row>
     <row r="30" ht="40.5" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
@@ -6467,10 +6576,11 @@
           <t>确认</t>
         </is>
       </c>
-      <c r="S30" s="2" t="inlineStr"/>
+      <c r="S30" s="9" t="n"/>
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="inlineStr"/>
+      <c r="W30" s="2" t="inlineStr"/>
     </row>
     <row r="31" ht="27" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
@@ -6539,14 +6649,15 @@
           <t>确认</t>
         </is>
       </c>
-      <c r="S31" s="5" t="inlineStr">
-        <is>
-          <t>确认</t>
-        </is>
-      </c>
-      <c r="T31" s="2" t="inlineStr"/>
+      <c r="S31" s="9" t="n"/>
+      <c r="T31" s="5" t="inlineStr">
+        <is>
+          <t>确认</t>
+        </is>
+      </c>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="inlineStr"/>
+      <c r="W31" s="2" t="inlineStr"/>
     </row>
     <row r="32" ht="27" customHeight="1">
       <c r="A32" s="3" t="inlineStr">
@@ -6615,14 +6726,15 @@
           <t>确认</t>
         </is>
       </c>
-      <c r="S32" s="5" t="inlineStr">
-        <is>
-          <t>确认</t>
-        </is>
-      </c>
-      <c r="T32" s="2" t="inlineStr"/>
+      <c r="S32" s="9" t="n"/>
+      <c r="T32" s="5" t="inlineStr">
+        <is>
+          <t>确认</t>
+        </is>
+      </c>
       <c r="U32" s="2" t="inlineStr"/>
       <c r="V32" s="2" t="inlineStr"/>
+      <c r="W32" s="2" t="inlineStr"/>
     </row>
     <row r="33" ht="27" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
@@ -6683,10 +6795,11 @@
       <c r="P33" s="2" t="inlineStr"/>
       <c r="Q33" s="2" t="inlineStr"/>
       <c r="R33" s="2" t="inlineStr"/>
-      <c r="S33" s="2" t="inlineStr"/>
+      <c r="S33" s="7" t="n"/>
       <c r="T33" s="2" t="inlineStr"/>
       <c r="U33" s="2" t="inlineStr"/>
       <c r="V33" s="2" t="inlineStr"/>
+      <c r="W33" s="2" t="inlineStr"/>
     </row>
     <row r="34" ht="27" customHeight="1">
       <c r="A34" s="3" t="inlineStr">
@@ -6747,10 +6860,11 @@
       <c r="P34" s="2" t="inlineStr"/>
       <c r="Q34" s="2" t="inlineStr"/>
       <c r="R34" s="2" t="inlineStr"/>
-      <c r="S34" s="2" t="inlineStr"/>
+      <c r="S34" s="7" t="n"/>
       <c r="T34" s="2" t="inlineStr"/>
       <c r="U34" s="2" t="inlineStr"/>
       <c r="V34" s="2" t="inlineStr"/>
+      <c r="W34" s="2" t="inlineStr"/>
     </row>
     <row r="35" ht="27" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
@@ -6811,10 +6925,11 @@
       <c r="P35" s="2" t="inlineStr"/>
       <c r="Q35" s="2" t="inlineStr"/>
       <c r="R35" s="2" t="inlineStr"/>
-      <c r="S35" s="2" t="inlineStr"/>
+      <c r="S35" s="7" t="n"/>
       <c r="T35" s="2" t="inlineStr"/>
       <c r="U35" s="2" t="inlineStr"/>
       <c r="V35" s="2" t="inlineStr"/>
+      <c r="W35" s="2" t="inlineStr"/>
     </row>
     <row r="36" ht="27" customHeight="1">
       <c r="A36" s="3" t="inlineStr">
@@ -6875,10 +6990,11 @@
       <c r="P36" s="2" t="inlineStr"/>
       <c r="Q36" s="2" t="inlineStr"/>
       <c r="R36" s="2" t="inlineStr"/>
-      <c r="S36" s="2" t="inlineStr"/>
+      <c r="S36" s="7" t="n"/>
       <c r="T36" s="2" t="inlineStr"/>
       <c r="U36" s="2" t="inlineStr"/>
       <c r="V36" s="2" t="inlineStr"/>
+      <c r="W36" s="2" t="inlineStr"/>
     </row>
     <row r="37" ht="27" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
@@ -6939,10 +7055,11 @@
       <c r="P37" s="2" t="inlineStr"/>
       <c r="Q37" s="2" t="inlineStr"/>
       <c r="R37" s="2" t="inlineStr"/>
-      <c r="S37" s="2" t="inlineStr"/>
+      <c r="S37" s="7" t="n"/>
       <c r="T37" s="2" t="inlineStr"/>
       <c r="U37" s="2" t="inlineStr"/>
       <c r="V37" s="2" t="inlineStr"/>
+      <c r="W37" s="2" t="inlineStr"/>
     </row>
     <row r="38" ht="27" customHeight="1">
       <c r="A38" s="3" t="inlineStr">
@@ -7003,10 +7120,11 @@
       <c r="P38" s="2" t="inlineStr"/>
       <c r="Q38" s="2" t="inlineStr"/>
       <c r="R38" s="2" t="inlineStr"/>
-      <c r="S38" s="2" t="inlineStr"/>
+      <c r="S38" s="7" t="n"/>
       <c r="T38" s="2" t="inlineStr"/>
       <c r="U38" s="2" t="inlineStr"/>
       <c r="V38" s="2" t="inlineStr"/>
+      <c r="W38" s="2" t="inlineStr"/>
     </row>
     <row r="39" ht="27" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
@@ -7067,10 +7185,11 @@
       <c r="P39" s="2" t="inlineStr"/>
       <c r="Q39" s="2" t="inlineStr"/>
       <c r="R39" s="2" t="inlineStr"/>
-      <c r="S39" s="2" t="inlineStr"/>
+      <c r="S39" s="7" t="n"/>
       <c r="T39" s="2" t="inlineStr"/>
       <c r="U39" s="2" t="inlineStr"/>
       <c r="V39" s="2" t="inlineStr"/>
+      <c r="W39" s="2" t="inlineStr"/>
     </row>
     <row r="40" ht="27" customHeight="1">
       <c r="A40" s="3" t="inlineStr">
@@ -7131,10 +7250,11 @@
       <c r="P40" s="2" t="inlineStr"/>
       <c r="Q40" s="2" t="inlineStr"/>
       <c r="R40" s="2" t="inlineStr"/>
-      <c r="S40" s="2" t="inlineStr"/>
+      <c r="S40" s="7" t="n"/>
       <c r="T40" s="2" t="inlineStr"/>
       <c r="U40" s="2" t="inlineStr"/>
       <c r="V40" s="2" t="inlineStr"/>
+      <c r="W40" s="2" t="inlineStr"/>
     </row>
     <row r="41" ht="27" customHeight="1">
       <c r="A41" s="3" t="inlineStr">
@@ -7195,10 +7315,11 @@
       <c r="P41" s="2" t="inlineStr"/>
       <c r="Q41" s="2" t="inlineStr"/>
       <c r="R41" s="2" t="inlineStr"/>
-      <c r="S41" s="2" t="inlineStr"/>
+      <c r="S41" s="7" t="n"/>
       <c r="T41" s="2" t="inlineStr"/>
       <c r="U41" s="2" t="inlineStr"/>
       <c r="V41" s="2" t="inlineStr"/>
+      <c r="W41" s="2" t="inlineStr"/>
     </row>
     <row r="42" ht="27" customHeight="1">
       <c r="A42" s="3" t="inlineStr">
@@ -7259,10 +7380,11 @@
       <c r="P42" s="2" t="inlineStr"/>
       <c r="Q42" s="2" t="inlineStr"/>
       <c r="R42" s="2" t="inlineStr"/>
-      <c r="S42" s="2" t="inlineStr"/>
+      <c r="S42" s="7" t="n"/>
       <c r="T42" s="2" t="inlineStr"/>
       <c r="U42" s="2" t="inlineStr"/>
       <c r="V42" s="2" t="inlineStr"/>
+      <c r="W42" s="2" t="inlineStr"/>
     </row>
     <row r="43" ht="27" customHeight="1">
       <c r="A43" s="3" t="inlineStr">
@@ -7323,10 +7445,11 @@
       <c r="P43" s="2" t="inlineStr"/>
       <c r="Q43" s="2" t="inlineStr"/>
       <c r="R43" s="2" t="inlineStr"/>
-      <c r="S43" s="2" t="inlineStr"/>
+      <c r="S43" s="7" t="n"/>
       <c r="T43" s="2" t="inlineStr"/>
       <c r="U43" s="2" t="inlineStr"/>
       <c r="V43" s="2" t="inlineStr"/>
+      <c r="W43" s="2" t="inlineStr"/>
     </row>
     <row r="44" ht="27" customHeight="1">
       <c r="A44" s="3" t="inlineStr">
@@ -7387,10 +7510,11 @@
       <c r="P44" s="2" t="inlineStr"/>
       <c r="Q44" s="2" t="inlineStr"/>
       <c r="R44" s="2" t="inlineStr"/>
-      <c r="S44" s="2" t="inlineStr"/>
+      <c r="S44" s="7" t="n"/>
       <c r="T44" s="2" t="inlineStr"/>
       <c r="U44" s="2" t="inlineStr"/>
       <c r="V44" s="2" t="inlineStr"/>
+      <c r="W44" s="2" t="inlineStr"/>
     </row>
     <row r="45" ht="27" customHeight="1">
       <c r="A45" s="3" t="inlineStr">
@@ -7451,10 +7575,11 @@
       <c r="P45" s="2" t="inlineStr"/>
       <c r="Q45" s="2" t="inlineStr"/>
       <c r="R45" s="2" t="inlineStr"/>
-      <c r="S45" s="2" t="inlineStr"/>
+      <c r="S45" s="7" t="n"/>
       <c r="T45" s="2" t="inlineStr"/>
       <c r="U45" s="2" t="inlineStr"/>
       <c r="V45" s="2" t="inlineStr"/>
+      <c r="W45" s="2" t="inlineStr"/>
     </row>
     <row r="46" ht="27" customHeight="1">
       <c r="A46" s="3" t="inlineStr">
@@ -7515,10 +7640,11 @@
       <c r="P46" s="2" t="inlineStr"/>
       <c r="Q46" s="2" t="inlineStr"/>
       <c r="R46" s="2" t="inlineStr"/>
-      <c r="S46" s="2" t="inlineStr"/>
+      <c r="S46" s="7" t="n"/>
       <c r="T46" s="2" t="inlineStr"/>
       <c r="U46" s="2" t="inlineStr"/>
       <c r="V46" s="2" t="inlineStr"/>
+      <c r="W46" s="2" t="inlineStr"/>
     </row>
     <row r="47" ht="27" customHeight="1">
       <c r="A47" s="3" t="inlineStr">
@@ -7579,10 +7705,11 @@
       <c r="P47" s="2" t="inlineStr"/>
       <c r="Q47" s="2" t="inlineStr"/>
       <c r="R47" s="2" t="inlineStr"/>
-      <c r="S47" s="2" t="inlineStr"/>
+      <c r="S47" s="7" t="n"/>
       <c r="T47" s="2" t="inlineStr"/>
       <c r="U47" s="2" t="inlineStr"/>
       <c r="V47" s="2" t="inlineStr"/>
+      <c r="W47" s="2" t="inlineStr"/>
     </row>
     <row r="48" ht="27" customHeight="1">
       <c r="A48" s="3" t="inlineStr">
@@ -7643,10 +7770,11 @@
       <c r="P48" s="2" t="inlineStr"/>
       <c r="Q48" s="2" t="inlineStr"/>
       <c r="R48" s="2" t="inlineStr"/>
-      <c r="S48" s="2" t="inlineStr"/>
+      <c r="S48" s="7" t="n"/>
       <c r="T48" s="2" t="inlineStr"/>
       <c r="U48" s="2" t="inlineStr"/>
       <c r="V48" s="2" t="inlineStr"/>
+      <c r="W48" s="2" t="inlineStr"/>
     </row>
     <row r="49" ht="27" customHeight="1">
       <c r="A49" s="3" t="inlineStr">
@@ -7707,10 +7835,11 @@
       <c r="P49" s="2" t="inlineStr"/>
       <c r="Q49" s="2" t="inlineStr"/>
       <c r="R49" s="2" t="inlineStr"/>
-      <c r="S49" s="2" t="inlineStr"/>
+      <c r="S49" s="7" t="n"/>
       <c r="T49" s="2" t="inlineStr"/>
       <c r="U49" s="2" t="inlineStr"/>
       <c r="V49" s="2" t="inlineStr"/>
+      <c r="W49" s="2" t="inlineStr"/>
     </row>
     <row r="50" ht="27" customHeight="1">
       <c r="A50" s="3" t="inlineStr">
@@ -7771,10 +7900,11 @@
       <c r="P50" s="2" t="inlineStr"/>
       <c r="Q50" s="2" t="inlineStr"/>
       <c r="R50" s="2" t="inlineStr"/>
-      <c r="S50" s="2" t="inlineStr"/>
+      <c r="S50" s="7" t="n"/>
       <c r="T50" s="2" t="inlineStr"/>
       <c r="U50" s="2" t="inlineStr"/>
       <c r="V50" s="2" t="inlineStr"/>
+      <c r="W50" s="2" t="inlineStr"/>
     </row>
     <row r="51" ht="27" customHeight="1">
       <c r="A51" s="3" t="inlineStr">
@@ -7835,10 +7965,11 @@
       <c r="P51" s="2" t="inlineStr"/>
       <c r="Q51" s="2" t="inlineStr"/>
       <c r="R51" s="2" t="inlineStr"/>
-      <c r="S51" s="2" t="inlineStr"/>
+      <c r="S51" s="7" t="n"/>
       <c r="T51" s="2" t="inlineStr"/>
       <c r="U51" s="2" t="inlineStr"/>
       <c r="V51" s="2" t="inlineStr"/>
+      <c r="W51" s="2" t="inlineStr"/>
     </row>
     <row r="52" ht="27" customHeight="1">
       <c r="A52" s="3" t="inlineStr">
@@ -7899,10 +8030,11 @@
       <c r="P52" s="2" t="inlineStr"/>
       <c r="Q52" s="2" t="inlineStr"/>
       <c r="R52" s="2" t="inlineStr"/>
-      <c r="S52" s="2" t="inlineStr"/>
+      <c r="S52" s="7" t="n"/>
       <c r="T52" s="2" t="inlineStr"/>
       <c r="U52" s="2" t="inlineStr"/>
       <c r="V52" s="2" t="inlineStr"/>
+      <c r="W52" s="2" t="inlineStr"/>
     </row>
     <row r="53" ht="40.5" customHeight="1">
       <c r="A53" s="3" t="inlineStr">
@@ -7963,18 +8095,19 @@
       <c r="P53" s="2" t="n"/>
       <c r="Q53" s="2" t="n"/>
       <c r="R53" s="2" t="n"/>
-      <c r="S53" s="2" t="n"/>
-      <c r="T53" s="5" t="inlineStr">
-        <is>
-          <t>确认</t>
-        </is>
-      </c>
+      <c r="S53" s="7" t="n"/>
+      <c r="T53" s="2" t="n"/>
       <c r="U53" s="5" t="inlineStr">
         <is>
           <t>确认</t>
         </is>
       </c>
-      <c r="V53" s="2" t="n"/>
+      <c r="V53" s="5" t="inlineStr">
+        <is>
+          <t>确认</t>
+        </is>
+      </c>
+      <c r="W53" s="2" t="n"/>
     </row>
     <row r="54" ht="27" customHeight="1">
       <c r="A54" s="3" t="inlineStr">
@@ -8027,10 +8160,11 @@
       <c r="P54" s="2" t="inlineStr"/>
       <c r="Q54" s="2" t="inlineStr"/>
       <c r="R54" s="2" t="inlineStr"/>
-      <c r="S54" s="2" t="inlineStr"/>
+      <c r="S54" s="7" t="n"/>
       <c r="T54" s="2" t="inlineStr"/>
       <c r="U54" s="2" t="inlineStr"/>
       <c r="V54" s="2" t="inlineStr"/>
+      <c r="W54" s="2" t="inlineStr"/>
     </row>
     <row r="55" ht="27" customHeight="1">
       <c r="A55" s="3" t="inlineStr">
@@ -8083,10 +8217,11 @@
       <c r="P55" s="2" t="inlineStr"/>
       <c r="Q55" s="2" t="inlineStr"/>
       <c r="R55" s="2" t="inlineStr"/>
-      <c r="S55" s="2" t="inlineStr"/>
+      <c r="S55" s="7" t="n"/>
       <c r="T55" s="2" t="inlineStr"/>
       <c r="U55" s="2" t="inlineStr"/>
-      <c r="V55" s="5" t="inlineStr">
+      <c r="V55" s="2" t="inlineStr"/>
+      <c r="W55" s="5" t="inlineStr">
         <is>
           <t>确认</t>
         </is>
@@ -8151,10 +8286,11 @@
       <c r="P56" s="2" t="inlineStr"/>
       <c r="Q56" s="2" t="inlineStr"/>
       <c r="R56" s="2" t="inlineStr"/>
-      <c r="S56" s="2" t="inlineStr"/>
+      <c r="S56" s="7" t="n"/>
       <c r="T56" s="2" t="inlineStr"/>
       <c r="U56" s="2" t="inlineStr"/>
       <c r="V56" s="2" t="inlineStr"/>
+      <c r="W56" s="2" t="inlineStr"/>
     </row>
     <row r="57" ht="27" customHeight="1">
       <c r="A57" s="3" t="inlineStr">
@@ -8215,10 +8351,11 @@
       <c r="P57" s="2" t="inlineStr"/>
       <c r="Q57" s="2" t="inlineStr"/>
       <c r="R57" s="2" t="inlineStr"/>
-      <c r="S57" s="2" t="inlineStr"/>
+      <c r="S57" s="7" t="n"/>
       <c r="T57" s="2" t="inlineStr"/>
       <c r="U57" s="2" t="inlineStr"/>
       <c r="V57" s="2" t="inlineStr"/>
+      <c r="W57" s="2" t="inlineStr"/>
     </row>
     <row r="58" ht="27" customHeight="1">
       <c r="A58" s="3" t="inlineStr">
@@ -8279,10 +8416,11 @@
       <c r="P58" s="2" t="inlineStr"/>
       <c r="Q58" s="2" t="inlineStr"/>
       <c r="R58" s="2" t="inlineStr"/>
-      <c r="S58" s="2" t="inlineStr"/>
+      <c r="S58" s="7" t="n"/>
       <c r="T58" s="2" t="inlineStr"/>
       <c r="U58" s="2" t="inlineStr"/>
       <c r="V58" s="2" t="inlineStr"/>
+      <c r="W58" s="2" t="inlineStr"/>
     </row>
     <row r="59" ht="27" customHeight="1">
       <c r="A59" s="3" t="inlineStr">
@@ -8343,10 +8481,11 @@
       <c r="P59" s="2" t="inlineStr"/>
       <c r="Q59" s="2" t="inlineStr"/>
       <c r="R59" s="2" t="inlineStr"/>
-      <c r="S59" s="2" t="inlineStr"/>
+      <c r="S59" s="7" t="n"/>
       <c r="T59" s="2" t="inlineStr"/>
       <c r="U59" s="2" t="inlineStr"/>
       <c r="V59" s="2" t="inlineStr"/>
+      <c r="W59" s="2" t="inlineStr"/>
     </row>
     <row r="60" ht="27" customHeight="1">
       <c r="A60" s="3" t="inlineStr">
@@ -8407,10 +8546,11 @@
       <c r="P60" s="2" t="inlineStr"/>
       <c r="Q60" s="2" t="inlineStr"/>
       <c r="R60" s="2" t="inlineStr"/>
-      <c r="S60" s="2" t="inlineStr"/>
+      <c r="S60" s="7" t="n"/>
       <c r="T60" s="2" t="inlineStr"/>
       <c r="U60" s="2" t="inlineStr"/>
       <c r="V60" s="2" t="inlineStr"/>
+      <c r="W60" s="2" t="inlineStr"/>
     </row>
     <row r="61" ht="27" customHeight="1">
       <c r="A61" s="3" t="inlineStr">
@@ -8471,10 +8611,11 @@
       <c r="P61" s="2" t="inlineStr"/>
       <c r="Q61" s="2" t="inlineStr"/>
       <c r="R61" s="2" t="inlineStr"/>
-      <c r="S61" s="2" t="inlineStr"/>
+      <c r="S61" s="7" t="n"/>
       <c r="T61" s="2" t="inlineStr"/>
       <c r="U61" s="2" t="inlineStr"/>
       <c r="V61" s="2" t="inlineStr"/>
+      <c r="W61" s="2" t="inlineStr"/>
     </row>
     <row r="62" ht="27" customHeight="1">
       <c r="A62" s="3" t="inlineStr">
@@ -8535,10 +8676,11 @@
       <c r="P62" s="2" t="inlineStr"/>
       <c r="Q62" s="2" t="inlineStr"/>
       <c r="R62" s="2" t="inlineStr"/>
-      <c r="S62" s="2" t="inlineStr"/>
+      <c r="S62" s="7" t="n"/>
       <c r="T62" s="2" t="inlineStr"/>
       <c r="U62" s="2" t="inlineStr"/>
       <c r="V62" s="2" t="inlineStr"/>
+      <c r="W62" s="2" t="inlineStr"/>
     </row>
     <row r="63" ht="27" customHeight="1">
       <c r="A63" s="3" t="inlineStr">
@@ -8599,10 +8741,11 @@
       <c r="P63" s="2" t="inlineStr"/>
       <c r="Q63" s="2" t="inlineStr"/>
       <c r="R63" s="2" t="inlineStr"/>
-      <c r="S63" s="2" t="inlineStr"/>
+      <c r="S63" s="7" t="n"/>
       <c r="T63" s="2" t="inlineStr"/>
       <c r="U63" s="2" t="inlineStr"/>
       <c r="V63" s="2" t="inlineStr"/>
+      <c r="W63" s="2" t="inlineStr"/>
     </row>
     <row r="64" ht="27" customHeight="1">
       <c r="A64" s="3" t="inlineStr">
@@ -8663,10 +8806,11 @@
       <c r="P64" s="2" t="inlineStr"/>
       <c r="Q64" s="2" t="inlineStr"/>
       <c r="R64" s="2" t="inlineStr"/>
-      <c r="S64" s="2" t="inlineStr"/>
+      <c r="S64" s="7" t="n"/>
       <c r="T64" s="2" t="inlineStr"/>
       <c r="U64" s="2" t="inlineStr"/>
       <c r="V64" s="2" t="inlineStr"/>
+      <c r="W64" s="2" t="inlineStr"/>
     </row>
     <row r="65" ht="27" customHeight="1">
       <c r="A65" s="3" t="inlineStr">
@@ -8727,10 +8871,11 @@
       <c r="P65" s="2" t="inlineStr"/>
       <c r="Q65" s="2" t="inlineStr"/>
       <c r="R65" s="2" t="inlineStr"/>
-      <c r="S65" s="2" t="inlineStr"/>
+      <c r="S65" s="7" t="n"/>
       <c r="T65" s="2" t="inlineStr"/>
       <c r="U65" s="2" t="inlineStr"/>
       <c r="V65" s="2" t="inlineStr"/>
+      <c r="W65" s="2" t="inlineStr"/>
     </row>
     <row r="66" ht="27" customHeight="1">
       <c r="A66" s="3" t="inlineStr">
@@ -8791,10 +8936,11 @@
       <c r="P66" s="2" t="inlineStr"/>
       <c r="Q66" s="2" t="inlineStr"/>
       <c r="R66" s="2" t="inlineStr"/>
-      <c r="S66" s="2" t="inlineStr"/>
+      <c r="S66" s="7" t="n"/>
       <c r="T66" s="2" t="inlineStr"/>
       <c r="U66" s="2" t="inlineStr"/>
       <c r="V66" s="2" t="inlineStr"/>
+      <c r="W66" s="2" t="inlineStr"/>
     </row>
     <row r="67" ht="27" customHeight="1">
       <c r="A67" s="3" t="inlineStr">
@@ -8855,10 +9001,11 @@
       <c r="P67" s="2" t="inlineStr"/>
       <c r="Q67" s="2" t="inlineStr"/>
       <c r="R67" s="2" t="inlineStr"/>
-      <c r="S67" s="2" t="inlineStr"/>
+      <c r="S67" s="7" t="n"/>
       <c r="T67" s="2" t="inlineStr"/>
       <c r="U67" s="2" t="inlineStr"/>
       <c r="V67" s="2" t="inlineStr"/>
+      <c r="W67" s="2" t="inlineStr"/>
     </row>
     <row r="68" ht="27" customHeight="1">
       <c r="A68" s="3" t="inlineStr">
@@ -8878,17 +9025,17 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>状态、位置、称重、液位、水位、平均密度、平均温度、频率、电容、X角、Y角、罐高</t>
+          <t>状态、位置、称重、温度、频率、电容、X角、Y角、RSSI</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>`debug_data`、`oil_measurement`、`water_measurement`、`density_distribution`、`height_measurement.current_real_height`</t>
+          <t>`debug_data.sensor_position`、`debug_data.current_weight`、`debug_data.temperature`、`debug_data.frequency`、`debug_data.water_capacitance_x10`、`debug_data.angle_x/y`、`wireless_pairing_status.rssi_valid/rssi`</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>各项按有效值分页显示，频率和电容可同时显示</t>
+          <t>CPU2 `CMD_ReadPartParams()` 每 1s 刷新部件参数，RSSI 快照按 5s 节流刷新；读取参数态的 X/Y 角不受 `bottom_detect_mode` 限制；不混用液位、水位、罐高等历史业务结果</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -8911,21 +9058,9 @@
           <t>确认</t>
         </is>
       </c>
-      <c r="K68" s="2" t="inlineStr">
-        <is>
-          <t>确认</t>
-        </is>
-      </c>
-      <c r="L68" s="2" t="inlineStr">
-        <is>
-          <t>确认</t>
-        </is>
-      </c>
-      <c r="M68" s="2" t="inlineStr">
-        <is>
-          <t>确认</t>
-        </is>
-      </c>
+      <c r="K68" s="2" t="n"/>
+      <c r="L68" s="2" t="n"/>
+      <c r="M68" s="2" t="n"/>
       <c r="N68" s="2" t="inlineStr">
         <is>
           <t>确认</t>
@@ -8951,7 +9086,7 @@
           <t>确认</t>
         </is>
       </c>
-      <c r="S68" s="2" t="inlineStr">
+      <c r="S68" s="7" t="inlineStr">
         <is>
           <t>确认</t>
         </is>
@@ -8959,6 +9094,7 @@
       <c r="T68" s="2" t="n"/>
       <c r="U68" s="2" t="n"/>
       <c r="V68" s="2" t="n"/>
+      <c r="W68" s="2" t="n"/>
     </row>
     <row r="69" ht="27" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
@@ -9019,10 +9155,11 @@
       <c r="P69" s="2" t="inlineStr"/>
       <c r="Q69" s="2" t="inlineStr"/>
       <c r="R69" s="2" t="inlineStr"/>
-      <c r="S69" s="2" t="inlineStr"/>
+      <c r="S69" s="7" t="n"/>
       <c r="T69" s="2" t="inlineStr"/>
       <c r="U69" s="2" t="inlineStr"/>
       <c r="V69" s="2" t="inlineStr"/>
+      <c r="W69" s="2" t="inlineStr"/>
     </row>
     <row r="70" ht="27" customHeight="1">
       <c r="A70" s="3" t="inlineStr">
@@ -9083,10 +9220,11 @@
       <c r="P70" s="2" t="inlineStr"/>
       <c r="Q70" s="2" t="inlineStr"/>
       <c r="R70" s="2" t="inlineStr"/>
-      <c r="S70" s="2" t="inlineStr"/>
+      <c r="S70" s="7" t="n"/>
       <c r="T70" s="2" t="inlineStr"/>
       <c r="U70" s="2" t="inlineStr"/>
       <c r="V70" s="2" t="inlineStr"/>
+      <c r="W70" s="2" t="inlineStr"/>
     </row>
     <row r="71" ht="27" customHeight="1">
       <c r="A71" s="3" t="inlineStr">
@@ -9147,10 +9285,11 @@
       <c r="P71" s="2" t="inlineStr"/>
       <c r="Q71" s="2" t="inlineStr"/>
       <c r="R71" s="2" t="inlineStr"/>
-      <c r="S71" s="2" t="inlineStr"/>
+      <c r="S71" s="7" t="n"/>
       <c r="T71" s="2" t="inlineStr"/>
       <c r="U71" s="2" t="inlineStr"/>
       <c r="V71" s="2" t="inlineStr"/>
+      <c r="W71" s="2" t="inlineStr"/>
     </row>
     <row r="72" ht="27" customHeight="1">
       <c r="A72" s="3" t="inlineStr">
@@ -9211,10 +9350,11 @@
       <c r="P72" s="2" t="inlineStr"/>
       <c r="Q72" s="2" t="inlineStr"/>
       <c r="R72" s="2" t="inlineStr"/>
-      <c r="S72" s="2" t="inlineStr"/>
+      <c r="S72" s="7" t="n"/>
       <c r="T72" s="2" t="inlineStr"/>
       <c r="U72" s="2" t="inlineStr"/>
       <c r="V72" s="2" t="inlineStr"/>
+      <c r="W72" s="2" t="inlineStr"/>
     </row>
     <row r="73" ht="27" customHeight="1">
       <c r="A73" s="3" t="inlineStr">
@@ -9275,10 +9415,11 @@
       <c r="P73" s="2" t="inlineStr"/>
       <c r="Q73" s="2" t="inlineStr"/>
       <c r="R73" s="2" t="inlineStr"/>
-      <c r="S73" s="2" t="inlineStr"/>
+      <c r="S73" s="7" t="n"/>
       <c r="T73" s="2" t="inlineStr"/>
       <c r="U73" s="2" t="inlineStr"/>
       <c r="V73" s="2" t="inlineStr"/>
+      <c r="W73" s="2" t="inlineStr"/>
     </row>
     <row r="74" ht="27" customHeight="1">
       <c r="A74" s="3" t="inlineStr">
@@ -9339,10 +9480,11 @@
       <c r="P74" s="2" t="inlineStr"/>
       <c r="Q74" s="2" t="inlineStr"/>
       <c r="R74" s="2" t="inlineStr"/>
-      <c r="S74" s="2" t="inlineStr"/>
+      <c r="S74" s="7" t="n"/>
       <c r="T74" s="2" t="inlineStr"/>
       <c r="U74" s="2" t="inlineStr"/>
       <c r="V74" s="2" t="inlineStr"/>
+      <c r="W74" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:V74"/>
@@ -9356,7 +9498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -9400,7 +9542,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>液位状态取 `oil_measurement.oil_level`；分布完成取 `density_distribution.Density_oil_level`；综合完成和读取参数完成取 `oil_measurement.oil_level`</t>
+          <t>液位状态取 `oil_measurement.oil_level`；分布完成取 `density_distribution.Density_oil_level`；综合完成取 `oil_measurement.oil_level`</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -9444,7 +9586,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>单点测量、单点监测或分布平均密度；LTD 密度分布测量中和读取参数完成显示 `density_distribution.average_density`</t>
+          <t>单点测量、单点监测或分布平均密度；LTD 密度分布测量中显示 `density_distribution.average_density`</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -9466,7 +9608,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>单点测量、单点监测或分布平均温度；LTD 密度分布测量中和读取参数完成显示 `density_distribution.average_temperature`</t>
+          <t>单点测量、单点监测或分布平均温度；LTD 密度分布测量中显示 `density_distribution.average_temperature`；读取参数完成显示 `debug_data.temperature`</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -9532,7 +9674,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>优先 `oil_measurement.current_frequency`，否则 `debug_data.frequency`</t>
+          <t>液位过程取 `oil_measurement.current_frequency` 或 `debug_data.frequency`；读取参数完成取 `debug_data.frequency`</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -9549,17 +9691,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>水位过程/水位跟随状态，或读取参数完成，且 `water_measurement.current_capacitance &gt; 0`</t>
+          <t>水位过程/水位跟随状态，或读取参数完成，且当前电容有效</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>`water_measurement.current_capacitance`</t>
+          <t>水位过程取 `water_measurement.current_capacitance`；读取参数完成取 `debug_data.water_capacitance_x10`</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>显示为 `current_capacitance * 10`，小数 1 位</t>
+          <t>显示为 0.1pF 口径，小数 1 位</t>
         </is>
       </c>
     </row>
@@ -9571,7 +9713,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>罐高上下文或读取参数完成，且 `bottom_detect_mode != 0`，角度不为 `0`</t>
+          <t>读取参数完成时只要求角度不为 `0`；罐高上下文仍要求 `bottom_detect_mode != 0` 且角度不为 `0`</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -9581,71 +9723,93 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>小数 2 位，单位 `°`</t>
+          <t>原始值为角度 `x100`，小数 2 位，单位 `°`</t>
         </is>
       </c>
     </row>
     <row r="11" ht="27" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>蓝牙 RSSI</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>读取参数完成；`rssi_valid != 0` 时显示数值，否则显示无有效值</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>`wireless_pairing_status.rssi_valid` / `wireless_pairing_status.rssi`</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>单位 `dB`，无效时显示 `RSSI:N/A`</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>罐高</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>罐底完成、罐高标定完成或读取参数完成，且 `current_real_height != 0`</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>罐底完成或罐高标定完成，且 `current_real_height != 0`</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>`height_measurement.current_real_height`</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>`0.1 mm`</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>错误码</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>`STATE_ERROR`</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>`device_status.error_code`</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>状态行追加错误类型和位置，格式为 `type-pos`</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
+          <t>错误码</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>`STATE_ERROR`</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>`device_status.error_code`</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>状态行追加错误类型和位置，格式为 `type-pos`</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
           <t>故障详情</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>`STATE_ERROR` 且 `error_code != NO_ERROR`</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>`Display_GetErrorReasonByCode(error_code)`</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>结果区显示 `故障:` 原因，过长时拆成两行</t>
         </is>
@@ -9663,7 +9827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="7"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -9778,6 +9942,18 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>更新记录</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-13：同步读取参数完成态，移除液位/水位/密度/罐高历史结果，新增蓝牙 RSSI，并修正读取参数态 X/Y 角不受探底模式限制。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>